<commit_message>
Include additional/fixed corrections from CH ~7Nov
</commit_message>
<xml_diff>
--- a/docs/from_CH/Exp1 Errors_Corrections_Template_26Oct2024.xlsx
+++ b/docs/from_CH/Exp1 Errors_Corrections_Template_26Oct2024.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3239" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="307">
   <si>
     <t xml:space="preserve">Ignore all CBF1 files- data will not be analysed</t>
   </si>
@@ -789,19 +789,19 @@
     <t xml:space="preserve">Experiment_2023-10-22T11:36:41.453331_bonnie_79_Test Type 1.log</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-13T06/36/50.258957_myrtle_2.0_Training - fixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-13T07/17/20.615404_yoshi_2.0_Training - fixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-13T08/28/59.797750_gio_2.0_Training - fixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-13T10/22/11.789817_dusty_2.0_Training - fixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-13T13/01/26.435669_clover_nan_Training - fixed</t>
+    <t xml:space="preserve">Experiment_2023-11-13T06:36:50.258957_myrtle_2.0_Training - fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-13T07:17:20.615404_yoshi_2.0_Training - fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-13T08:28:59.797750_gio_2.0_Training - fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-13T10:22:11.789817_dusty_2.0_Training - fixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-13T13:01:26.435669_clover_nan_Training - fixed</t>
   </si>
   <si>
     <t xml:space="preserve">N </t>
@@ -810,73 +810,76 @@
     <t xml:space="preserve">Check if NOGO</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-13T16/34/23.409480_nix_3.0_Training randomised Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-13T17/24/29.152222_gio_3.0_Training randomised Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-13T18/03/46.698927_dusty_3.0_Training randomised Type 1</t>
+    <t xml:space="preserve">Experiment_2023-11-13T16:34:23.409480_nix_3.0_Training randomised Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-13T17:24:29.152222_gio_3.0_Training randomised Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-13T18:03:46.698927_dusty_3.0_Training randomised Type 1</t>
   </si>
   <si>
     <t xml:space="preserve">Go response- wrong buckets-extrapolated</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-13T20/54/16.427672_clover_nan_Training randomised Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T00/45/14.508317_myrtle_4.0_Training randomised Type 2</t>
+    <t xml:space="preserve">Experiment_2023-11-13T20:54:16.427672_clover_nan_Training randomised Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T00:45:14.508317_myrtle_4.0_Training randomised Type 2</t>
   </si>
   <si>
     <t xml:space="preserve">Note combine two files</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-14T01/18/45.941991_myrtle_5.0_Training randomised Type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T04/07/06.316598_gio_4.0_Training randomised Type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T10/23/47.643202_myrtle_6.0_Training randomised Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T12/13/40.543722_dusty_6.0_Training randomised Type 1</t>
+    <t xml:space="preserve">Experiment_2023-11-14T01:18:45.941991_myrtle_5.0_Training randomised Type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T04:07:06.316598_gio_4.0_Training randomised Type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should be NULL ResponseType  - leave blank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T10:23:47.643202_myrtle_6.0_Training randomised Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T12:13:40.543722_dusty_6.0_Training randomised Type 1</t>
   </si>
   <si>
     <t xml:space="preserve">Change session ID on MB's file</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-14T12/37/30.469954_gio_5.0_Test Type 1</t>
+    <t xml:space="preserve">Experiment_2023-11-14T12:37:30.469954_gio_5.0_Test Type 1</t>
   </si>
   <si>
     <t xml:space="preserve">Pumba</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-14T15/40/26.284336_pumba_nan_Training randomised Type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T17/14/25.139579_jelly_6.0_Test Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T18/48/28.476282_myrtle_8.0_Test Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-14T19/16/58.918521_yoshi_6.0_Training randomised Type 1</t>
+    <t xml:space="preserve">Experiment_2023-11-14T15:40:26.284336_pumba_nan_Training randomised Type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T17:14:25.139579_jelly_6.0_Test Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T18:48:28.476282_myrtle_8.0_Test Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-14T19:16:58.918521_yoshi_6.0_Training randomised Type 1</t>
   </si>
   <si>
     <t xml:space="preserve">Keep original values</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-14T23/17/57.967289_freya_nan_Test Type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-15T02/59/50.231712_george_6.0_Test Type 2</t>
+    <t xml:space="preserve">Experiment_2023-11-14T23:17:57.967289_freya_nan_Test Type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-15T02:59:50.231712_george_6.0_Test Type 2</t>
   </si>
   <si>
     <t xml:space="preserve"> Errors in test- 7N + 5P</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-15T04/42/42.109160_nix_9.0_Test Type 1</t>
+    <t xml:space="preserve">Experiment_2023-11-15T04:42:42.109160_nix_9.0_Test Type 1</t>
   </si>
   <si>
     <t xml:space="preserve">Meant to be P</t>
@@ -891,52 +894,52 @@
     <t xml:space="preserve">meant to be P</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-15T05/22/53.513691_gio_6.0_Test Type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-15T16/42/36.211643_smudge_8.0_Test Type 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-15T18/35/59.371714_yoshi_9.0_Test Type 2</t>
+    <t xml:space="preserve">Experiment_2023-11-15T05:22:53.513691_gio_6.0_Test Type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-15T16:42:36.211643_smudge_8.0_Test Type 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-15T18:35:59.371714_yoshi_9.0_Test Type 2</t>
   </si>
   <si>
     <t xml:space="preserve">Errors in test at trial 11 a N was run instead of a P.  An extra trial was added so horse did 16 trials</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-15T23/18/27.463685_clover_nan_Test Type 2</t>
+    <t xml:space="preserve">Experiment_2023-11-15T23:18:27.463685_clover_nan_Test Type 2</t>
   </si>
   <si>
     <t xml:space="preserve">Was run as N, then repeated so horse did extra 11 (P). </t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-16T09/12/31.465402_nix_10.0_Test Type 3</t>
+    <t xml:space="preserve">Experiment_2023-11-16T09:12:31.465402_nix_10.0_Test Type 3</t>
   </si>
   <si>
     <t xml:space="preserve">Two buckets (extra trial?)</t>
   </si>
   <si>
-    <t xml:space="preserve">Experiment_2023-11-16T15/46/42.899255_nix_11.0_Test Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-16T17/55/24.333022_gio_9.0_Test Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-16T19/24/59.492473_jelly_9.0_Test Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-16T20/27/00.214523_smudge_10.0_Test Type 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-16T21/17/46.006067_myrtle_10.0_Test Type 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-16T22/01/25.798273_yoshi_10.0_Test Type 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-16T23/55/33.357304_dusty_9.0_Test Type 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiment_2023-11-17T04/05/53.213724_dusty_10.0_Test Type 1</t>
+    <t xml:space="preserve">Experiment_2023-11-16T15:46:42.899255_nix_11.0_Test Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-16T17:55:24.333022_gio_9.0_Test Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-16T19:24:59.492473_jelly_9.0_Test Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-16T20:27:00.214523_smudge_10.0_Test Type 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-16T21:17:46.006067_myrtle_10.0_Test Type 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-16T22:01:25.798273_yoshi_10.0_Test Type 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-16T23:55:33.357304_dusty_9.0_Test Type 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiment_2023-11-17T04:05:53.213724_dusty_10.0_Test Type 1</t>
   </si>
   <si>
     <t xml:space="preserve">Bucket on the wrong side- was N, should have been P</t>
@@ -1025,7 +1028,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1035,7 +1038,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEEEEE"/>
-        <bgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -1058,8 +1061,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF81D41A"/>
+        <bgColor rgb="FF84E291"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFA6"/>
+        <bgColor rgb="FFFFFF6D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.5998"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <bgColor rgb="FF81D41A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF6D"/>
+        <bgColor rgb="FFFFFFA6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1153,7 +1174,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="57">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1334,7 +1355,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1346,19 +1367,35 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1375,6 +1412,79 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF8E86AE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEEEEE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF84E291"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF81D41A"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF6D"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFA6"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1395,7 +1505,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFFF6D"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -1412,14 +1522,14 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFFFA6"/>
       <rgbColor rgb="FF84E291"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FF81D41A"/>
       <rgbColor rgb="FFFFBF00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
@@ -2352,8 +2462,8 @@
       <c r="G50" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H50" s="0"/>
-      <c r="I50" s="0"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D51" s="3" t="n">
@@ -2377,8 +2487,8 @@
       <c r="G52" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H52" s="0"/>
-      <c r="I52" s="0"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
     </row>
     <row r="53" s="9" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="2"/>
@@ -2488,8 +2598,8 @@
       <c r="G59" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="H59" s="0"/>
-      <c r="I59" s="0"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D60" s="3" t="n">
@@ -2553,8 +2663,8 @@
       <c r="G64" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="H64" s="0"/>
-      <c r="I64" s="0"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D65" s="3" t="n">
@@ -2727,8 +2837,8 @@
       <c r="G76" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="H76" s="0"/>
-      <c r="I76" s="0"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="n">
@@ -2764,8 +2874,8 @@
       <c r="G78" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H78" s="0"/>
-      <c r="I78" s="0"/>
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="9"/>
@@ -2848,8 +2958,8 @@
       <c r="G83" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H83" s="0"/>
-      <c r="I83" s="0"/>
+      <c r="H83" s="11"/>
+      <c r="I83" s="11"/>
     </row>
     <row r="84" s="9" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1"/>
@@ -3118,8 +3228,8 @@
       <c r="G100" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H100" s="0"/>
-      <c r="I100" s="0"/>
+      <c r="H100" s="11"/>
+      <c r="I100" s="11"/>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="D101" s="3" t="n">
@@ -3215,8 +3325,8 @@
       <c r="G107" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="H107" s="0"/>
-      <c r="I107" s="0"/>
+      <c r="H107" s="11"/>
+      <c r="I107" s="11"/>
     </row>
     <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="12" t="n">
@@ -3248,8 +3358,8 @@
       <c r="G109" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="H109" s="0"/>
-      <c r="I109" s="0"/>
+      <c r="H109" s="11"/>
+      <c r="I109" s="11"/>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="12" t="n">
@@ -3432,8 +3542,8 @@
       <c r="G121" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H121" s="0"/>
-      <c r="I121" s="0"/>
+      <c r="H121" s="11"/>
+      <c r="I121" s="11"/>
     </row>
     <row r="122" s="9" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B122" s="2"/>
@@ -9905,7 +10015,9 @@
       <c r="F45" s="44" t="n">
         <v>9.35</v>
       </c>
-      <c r="G45" s="45"/>
+      <c r="G45" s="45" t="s">
+        <v>211</v>
+      </c>
       <c r="H45" s="44"/>
       <c r="I45" s="44" t="s">
         <v>136</v>
@@ -9925,7 +10037,7 @@
       </c>
       <c r="O45" s="47" t="str">
         <f aca="false">CONCATENATE(G45,", ",F45)</f>
-        <v>, 9.35</v>
+        <v>GO, 9.35</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9947,9 +10059,11 @@
       <c r="F46" s="31" t="n">
         <v>9.15</v>
       </c>
-      <c r="G46" s="41"/>
+      <c r="G46" s="48"/>
       <c r="H46" s="31"/>
-      <c r="I46" s="31"/>
+      <c r="I46" s="31" t="s">
+        <v>268</v>
+      </c>
       <c r="J46" s="39" t="s">
         <v>267</v>
       </c>
@@ -9986,9 +10100,11 @@
       <c r="F47" s="31" t="n">
         <v>9.01</v>
       </c>
-      <c r="G47" s="41"/>
+      <c r="G47" s="48"/>
       <c r="H47" s="31"/>
-      <c r="I47" s="31"/>
+      <c r="I47" s="31" t="s">
+        <v>268</v>
+      </c>
       <c r="J47" s="39" t="s">
         <v>267</v>
       </c>
@@ -10025,7 +10141,9 @@
       <c r="F48" s="31" t="n">
         <v>8.95</v>
       </c>
-      <c r="G48" s="41"/>
+      <c r="G48" s="45" t="s">
+        <v>211</v>
+      </c>
       <c r="H48" s="31"/>
       <c r="I48" s="31"/>
       <c r="J48" s="39" t="s">
@@ -10042,7 +10160,7 @@
       </c>
       <c r="O48" s="32" t="str">
         <f aca="false">CONCATENATE(G48,", ",F48)</f>
-        <v>, 8.95</v>
+        <v>GO, 8.95</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10146,9 +10264,11 @@
       <c r="F51" s="31" t="n">
         <v>8.69</v>
       </c>
-      <c r="G51" s="41"/>
+      <c r="G51" s="48"/>
       <c r="H51" s="31"/>
-      <c r="I51" s="31"/>
+      <c r="I51" s="31" t="s">
+        <v>268</v>
+      </c>
       <c r="J51" s="39" t="s">
         <v>267</v>
       </c>
@@ -10267,7 +10387,9 @@
       <c r="F54" s="31" t="n">
         <v>9.09</v>
       </c>
-      <c r="G54" s="41"/>
+      <c r="G54" s="45" t="s">
+        <v>211</v>
+      </c>
       <c r="H54" s="31"/>
       <c r="I54" s="31"/>
       <c r="J54" s="39" t="s">
@@ -10284,7 +10406,7 @@
       </c>
       <c r="O54" s="32" t="str">
         <f aca="false">CONCATENATE(G54,", ",F54)</f>
-        <v>, 9.09</v>
+        <v>GO, 9.09</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10347,7 +10469,9 @@
       <c r="F56" s="31" t="n">
         <v>9.13</v>
       </c>
-      <c r="G56" s="41"/>
+      <c r="G56" s="45" t="s">
+        <v>211</v>
+      </c>
       <c r="H56" s="31"/>
       <c r="I56" s="31"/>
       <c r="J56" s="39" t="s">
@@ -10364,7 +10488,7 @@
       </c>
       <c r="O56" s="32" t="str">
         <f aca="false">CONCATENATE(G56,", ",F56)</f>
-        <v>, 9.13</v>
+        <v>GO, 9.13</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10394,7 +10518,7 @@
         <v>20</v>
       </c>
       <c r="J57" s="39" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L57" s="31" t="s">
         <v>213</v>
@@ -10437,10 +10561,10 @@
         <v>39</v>
       </c>
       <c r="J58" s="42" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="K58" s="42" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L58" s="31" t="s">
         <v>213</v>
@@ -10483,7 +10607,7 @@
         <v>54</v>
       </c>
       <c r="J59" s="39" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L59" s="31" t="s">
         <v>213</v>
@@ -10526,7 +10650,7 @@
         <v>20</v>
       </c>
       <c r="J60" s="39" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L60" s="31" t="s">
         <v>213</v>
@@ -10569,7 +10693,7 @@
         <v>20</v>
       </c>
       <c r="J61" s="39" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="L61" s="31" t="s">
         <v>213</v>
@@ -10612,7 +10736,7 @@
         <v>149</v>
       </c>
       <c r="J62" s="39" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="L62" s="31" t="s">
         <v>213</v>
@@ -10636,7 +10760,7 @@
         <v>57</v>
       </c>
       <c r="C63" s="31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D63" s="31" t="n">
         <v>9</v>
@@ -10655,7 +10779,7 @@
         <v>152</v>
       </c>
       <c r="J63" s="39" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="L63" s="31" t="s">
         <v>213</v>
@@ -10685,14 +10809,18 @@
         <v>1</v>
       </c>
       <c r="E64" s="31"/>
-      <c r="F64" s="31"/>
-      <c r="G64" s="41"/>
+      <c r="F64" s="49" t="n">
+        <v>30</v>
+      </c>
+      <c r="G64" s="45" t="s">
+        <v>217</v>
+      </c>
       <c r="H64" s="31"/>
       <c r="I64" s="31" t="s">
         <v>154</v>
       </c>
       <c r="J64" s="39" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L64" s="31" t="s">
         <v>213</v>
@@ -10705,7 +10833,7 @@
       </c>
       <c r="O64" s="32" t="str">
         <f aca="false">CONCATENATE(G64,", ",F64)</f>
-        <v>, </v>
+        <v>NOGO, 30</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10735,7 +10863,7 @@
         <v>155</v>
       </c>
       <c r="J65" s="39" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="L65" s="31" t="s">
         <v>213</v>
@@ -10755,32 +10883,32 @@
       <c r="A66" s="30" t="n">
         <v>45250</v>
       </c>
-      <c r="B66" s="48" t="s">
+      <c r="B66" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="C66" s="48" t="s">
+      <c r="C66" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="D66" s="48" t="n">
+      <c r="D66" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="E66" s="48" t="s">
+      <c r="E66" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="F66" s="48" t="n">
+      <c r="F66" s="50" t="n">
         <v>9.68</v>
       </c>
-      <c r="G66" s="49" t="s">
-        <v>211</v>
-      </c>
-      <c r="H66" s="48"/>
-      <c r="I66" s="48" t="s">
+      <c r="G66" s="51" t="s">
+        <v>211</v>
+      </c>
+      <c r="H66" s="50"/>
+      <c r="I66" s="50" t="s">
         <v>156</v>
       </c>
-      <c r="J66" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="K66" s="50"/>
+      <c r="J66" s="52" t="s">
+        <v>277</v>
+      </c>
+      <c r="K66" s="52"/>
       <c r="L66" s="31" t="s">
         <v>213</v>
       </c>
@@ -10799,32 +10927,32 @@
       <c r="A67" s="30" t="n">
         <v>45250</v>
       </c>
-      <c r="B67" s="48" t="s">
+      <c r="B67" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="C67" s="48" t="s">
+      <c r="C67" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="D67" s="48" t="n">
+      <c r="D67" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="E67" s="48" t="s">
-        <v>14</v>
-      </c>
-      <c r="F67" s="48" t="n">
+      <c r="E67" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" s="50" t="n">
         <v>30</v>
       </c>
-      <c r="G67" s="49" t="s">
+      <c r="G67" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="H67" s="48"/>
-      <c r="I67" s="48" t="s">
+      <c r="H67" s="50"/>
+      <c r="I67" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="J67" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="K67" s="50"/>
+      <c r="J67" s="52" t="s">
+        <v>277</v>
+      </c>
+      <c r="K67" s="52"/>
       <c r="L67" s="31" t="s">
         <v>213</v>
       </c>
@@ -10843,32 +10971,32 @@
       <c r="A68" s="30" t="n">
         <v>45250</v>
       </c>
-      <c r="B68" s="48" t="s">
+      <c r="B68" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="C68" s="48" t="s">
+      <c r="C68" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="D68" s="48" t="n">
+      <c r="D68" s="50" t="n">
         <v>7</v>
       </c>
-      <c r="E68" s="48" t="s">
+      <c r="E68" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="F68" s="48" t="n">
+      <c r="F68" s="50" t="n">
         <v>30</v>
       </c>
-      <c r="G68" s="49" t="s">
+      <c r="G68" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="H68" s="48"/>
-      <c r="I68" s="48" t="s">
+      <c r="H68" s="50"/>
+      <c r="I68" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="J68" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="K68" s="50"/>
+      <c r="J68" s="52" t="s">
+        <v>277</v>
+      </c>
+      <c r="K68" s="52"/>
       <c r="L68" s="31" t="s">
         <v>213</v>
       </c>
@@ -10887,29 +11015,29 @@
       <c r="A69" s="30" t="n">
         <v>45250</v>
       </c>
-      <c r="B69" s="48" t="s">
+      <c r="B69" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="C69" s="48" t="s">
+      <c r="C69" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="D69" s="48" t="n">
+      <c r="D69" s="50" t="n">
         <v>8</v>
       </c>
-      <c r="E69" s="48" t="s">
-        <v>14</v>
-      </c>
-      <c r="F69" s="48"/>
-      <c r="G69" s="49"/>
-      <c r="H69" s="48"/>
-      <c r="I69" s="48" t="s">
+      <c r="E69" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F69" s="53"/>
+      <c r="G69" s="54"/>
+      <c r="H69" s="50"/>
+      <c r="I69" s="50" t="s">
         <v>157</v>
       </c>
-      <c r="J69" s="50" t="s">
-        <v>276</v>
-      </c>
-      <c r="K69" s="50" t="s">
+      <c r="J69" s="52" t="s">
         <v>277</v>
+      </c>
+      <c r="K69" s="52" t="s">
+        <v>278</v>
       </c>
       <c r="L69" s="31" t="s">
         <v>213</v>
@@ -10952,7 +11080,7 @@
         <v>159</v>
       </c>
       <c r="J70" s="39" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L70" s="31" t="s">
         <v>213</v>
@@ -10995,7 +11123,7 @@
         <v>20</v>
       </c>
       <c r="J71" s="39" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="L71" s="31" t="s">
         <v>213</v>
@@ -11035,10 +11163,10 @@
       </c>
       <c r="H72" s="31"/>
       <c r="I72" s="31" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J72" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L72" s="31" t="s">
         <v>213</v>
@@ -11079,7 +11207,7 @@
       <c r="H73" s="31"/>
       <c r="I73" s="31"/>
       <c r="J73" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L73" s="31" t="s">
         <v>213</v>
@@ -11120,7 +11248,7 @@
       <c r="H74" s="31"/>
       <c r="I74" s="31"/>
       <c r="J74" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L74" s="31" t="s">
         <v>213</v>
@@ -11160,10 +11288,10 @@
       </c>
       <c r="H75" s="31"/>
       <c r="I75" s="31" t="s">
+        <v>283</v>
+      </c>
+      <c r="J75" s="39" t="s">
         <v>282</v>
-      </c>
-      <c r="J75" s="39" t="s">
-        <v>281</v>
       </c>
       <c r="L75" s="31" t="s">
         <v>213</v>
@@ -11203,10 +11331,10 @@
       </c>
       <c r="H76" s="31"/>
       <c r="I76" s="31" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J76" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L76" s="31" t="s">
         <v>213</v>
@@ -11247,7 +11375,7 @@
       <c r="H77" s="31"/>
       <c r="I77" s="31"/>
       <c r="J77" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L77" s="31" t="s">
         <v>213</v>
@@ -11287,10 +11415,10 @@
       </c>
       <c r="H78" s="31"/>
       <c r="I78" s="31" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="J78" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L78" s="31" t="s">
         <v>213</v>
@@ -11330,10 +11458,10 @@
       </c>
       <c r="H79" s="31"/>
       <c r="I79" s="31" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="J79" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L79" s="31" t="s">
         <v>213</v>
@@ -11373,10 +11501,10 @@
       </c>
       <c r="H80" s="31"/>
       <c r="I80" s="31" t="s">
+        <v>283</v>
+      </c>
+      <c r="J80" s="39" t="s">
         <v>282</v>
-      </c>
-      <c r="J80" s="39" t="s">
-        <v>281</v>
       </c>
       <c r="L80" s="31" t="s">
         <v>213</v>
@@ -11416,10 +11544,10 @@
       </c>
       <c r="H81" s="31"/>
       <c r="I81" s="31" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="J81" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L81" s="31" t="s">
         <v>213</v>
@@ -11460,7 +11588,7 @@
       <c r="H82" s="31"/>
       <c r="I82" s="31"/>
       <c r="J82" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L82" s="31" t="s">
         <v>213</v>
@@ -11501,7 +11629,7 @@
       <c r="H83" s="31"/>
       <c r="I83" s="31"/>
       <c r="J83" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L83" s="31" t="s">
         <v>213</v>
@@ -11542,7 +11670,7 @@
       <c r="H84" s="31"/>
       <c r="I84" s="31"/>
       <c r="J84" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L84" s="31" t="s">
         <v>213</v>
@@ -11558,7 +11686,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="85" s="51" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="85" s="55" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11583,7 +11711,7 @@
       <c r="H85" s="31"/>
       <c r="I85" s="31"/>
       <c r="J85" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K85" s="39"/>
       <c r="L85" s="31" t="s">
@@ -11600,7 +11728,7 @@
         <v>GO, 11.09</v>
       </c>
     </row>
-    <row r="86" s="51" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="86" s="55" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11625,7 +11753,7 @@
       <c r="H86" s="31"/>
       <c r="I86" s="31"/>
       <c r="J86" s="39" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="K86" s="39"/>
       <c r="L86" s="31" t="s">
@@ -11642,7 +11770,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="87" s="51" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="87" s="55" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11669,7 +11797,7 @@
         <v>164</v>
       </c>
       <c r="J87" s="39" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K87" s="39"/>
       <c r="L87" s="31" t="s">
@@ -11686,7 +11814,7 @@
         <v>GO, 10.12</v>
       </c>
     </row>
-    <row r="88" s="51" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" s="55" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11713,7 +11841,7 @@
         <v>150</v>
       </c>
       <c r="J88" s="39" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="K88" s="39"/>
       <c r="L88" s="31" t="s">
@@ -11757,7 +11885,7 @@
         <v>167</v>
       </c>
       <c r="J89" s="39" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="L89" s="31" t="s">
         <v>213</v>
@@ -11792,13 +11920,15 @@
       <c r="F90" s="31" t="n">
         <v>10.93</v>
       </c>
-      <c r="G90" s="41"/>
+      <c r="G90" s="45" t="s">
+        <v>211</v>
+      </c>
       <c r="H90" s="31"/>
       <c r="I90" s="31" t="s">
         <v>54</v>
       </c>
       <c r="J90" s="39" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L90" s="31" t="s">
         <v>213</v>
@@ -11811,7 +11941,7 @@
       </c>
       <c r="O90" s="32" t="str">
         <f aca="false">CONCATENATE(G90,", ",F90)</f>
-        <v>, 10.93</v>
+        <v>GO, 10.93</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11838,10 +11968,10 @@
       </c>
       <c r="H91" s="31"/>
       <c r="I91" s="31" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="J91" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L91" s="31" t="s">
         <v>213</v>
@@ -11882,7 +12012,7 @@
       <c r="H92" s="31"/>
       <c r="I92" s="31"/>
       <c r="J92" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L92" s="31" t="s">
         <v>213</v>
@@ -11923,7 +12053,7 @@
       <c r="H93" s="31"/>
       <c r="I93" s="31"/>
       <c r="J93" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L93" s="31" t="s">
         <v>213</v>
@@ -11964,7 +12094,7 @@
       <c r="H94" s="31"/>
       <c r="I94" s="31"/>
       <c r="J94" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L94" s="31" t="s">
         <v>213</v>
@@ -12005,7 +12135,7 @@
       <c r="H95" s="31"/>
       <c r="I95" s="31"/>
       <c r="J95" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L95" s="31" t="s">
         <v>213</v>
@@ -12046,7 +12176,7 @@
       <c r="H96" s="31"/>
       <c r="I96" s="31"/>
       <c r="J96" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L96" s="31" t="s">
         <v>213</v>
@@ -12087,7 +12217,7 @@
       <c r="H97" s="31"/>
       <c r="I97" s="31"/>
       <c r="J97" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L97" s="31" t="s">
         <v>213</v>
@@ -12128,7 +12258,7 @@
       <c r="H98" s="31"/>
       <c r="I98" s="31"/>
       <c r="J98" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L98" s="31" t="s">
         <v>213</v>
@@ -12169,7 +12299,7 @@
       <c r="H99" s="31"/>
       <c r="I99" s="31"/>
       <c r="J99" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L99" s="31" t="s">
         <v>213</v>
@@ -12210,7 +12340,7 @@
       <c r="H100" s="31"/>
       <c r="I100" s="31"/>
       <c r="J100" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L100" s="31" t="s">
         <v>213</v>
@@ -12250,10 +12380,10 @@
       </c>
       <c r="H101" s="31"/>
       <c r="I101" s="31" t="s">
+        <v>292</v>
+      </c>
+      <c r="J101" s="39" t="s">
         <v>291</v>
-      </c>
-      <c r="J101" s="39" t="s">
-        <v>290</v>
       </c>
       <c r="L101" s="31" t="s">
         <v>213</v>
@@ -12294,7 +12424,7 @@
       <c r="H102" s="31"/>
       <c r="I102" s="31"/>
       <c r="J102" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L102" s="31" t="s">
         <v>213</v>
@@ -12335,7 +12465,7 @@
       <c r="H103" s="31"/>
       <c r="I103" s="31"/>
       <c r="J103" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L103" s="31" t="s">
         <v>213</v>
@@ -12376,7 +12506,7 @@
       <c r="H104" s="31"/>
       <c r="I104" s="31"/>
       <c r="J104" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L104" s="31" t="s">
         <v>213</v>
@@ -12417,7 +12547,7 @@
       <c r="H105" s="31"/>
       <c r="I105" s="31"/>
       <c r="J105" s="39" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L105" s="31" t="s">
         <v>213</v>
@@ -12460,7 +12590,7 @@
         <v>172</v>
       </c>
       <c r="J106" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L106" s="31" t="s">
         <v>213</v>
@@ -12501,7 +12631,7 @@
       <c r="H107" s="31"/>
       <c r="I107" s="31"/>
       <c r="J107" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L107" s="31" t="s">
         <v>213</v>
@@ -12542,7 +12672,7 @@
       <c r="H108" s="31"/>
       <c r="I108" s="31"/>
       <c r="J108" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L108" s="31" t="s">
         <v>213</v>
@@ -12583,7 +12713,7 @@
       <c r="H109" s="31"/>
       <c r="I109" s="31"/>
       <c r="J109" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L109" s="31" t="s">
         <v>213</v>
@@ -12624,7 +12754,7 @@
       <c r="H110" s="31"/>
       <c r="I110" s="31"/>
       <c r="J110" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L110" s="31" t="s">
         <v>213</v>
@@ -12665,7 +12795,7 @@
       <c r="H111" s="31"/>
       <c r="I111" s="31"/>
       <c r="J111" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L111" s="31" t="s">
         <v>213</v>
@@ -12708,7 +12838,7 @@
         <v>173</v>
       </c>
       <c r="J112" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L112" s="31" t="s">
         <v>213</v>
@@ -12748,10 +12878,10 @@
       </c>
       <c r="H113" s="31"/>
       <c r="I113" s="31" t="s">
+        <v>294</v>
+      </c>
+      <c r="J113" s="39" t="s">
         <v>293</v>
-      </c>
-      <c r="J113" s="39" t="s">
-        <v>292</v>
       </c>
       <c r="L113" s="31" t="s">
         <v>213</v>
@@ -12792,7 +12922,7 @@
       <c r="H114" s="31"/>
       <c r="I114" s="31"/>
       <c r="J114" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L114" s="31" t="s">
         <v>213</v>
@@ -12833,7 +12963,7 @@
       <c r="H115" s="31"/>
       <c r="I115" s="31"/>
       <c r="J115" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L115" s="31" t="s">
         <v>213</v>
@@ -12874,7 +13004,7 @@
       <c r="H116" s="31"/>
       <c r="I116" s="31"/>
       <c r="J116" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L116" s="31" t="s">
         <v>213</v>
@@ -12915,7 +13045,7 @@
       <c r="H117" s="31"/>
       <c r="I117" s="31"/>
       <c r="J117" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L117" s="31" t="s">
         <v>213</v>
@@ -12956,7 +13086,7 @@
       <c r="H118" s="31"/>
       <c r="I118" s="31"/>
       <c r="J118" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L118" s="31" t="s">
         <v>213</v>
@@ -12999,7 +13129,7 @@
         <v>174</v>
       </c>
       <c r="J119" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L119" s="31" t="s">
         <v>213</v>
@@ -13042,7 +13172,7 @@
         <v>54</v>
       </c>
       <c r="J120" s="39" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L120" s="31" t="s">
         <v>213</v>
@@ -13083,7 +13213,7 @@
       <c r="H121" s="31"/>
       <c r="I121" s="31"/>
       <c r="J121" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L121" s="31" t="s">
         <v>213</v>
@@ -13126,7 +13256,7 @@
         <v>20</v>
       </c>
       <c r="J122" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L122" s="31" t="s">
         <v>213</v>
@@ -13167,7 +13297,7 @@
       <c r="H123" s="31"/>
       <c r="I123" s="31"/>
       <c r="J123" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L123" s="31" t="s">
         <v>213</v>
@@ -13210,7 +13340,7 @@
         <v>182</v>
       </c>
       <c r="J124" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L124" s="31" t="s">
         <v>213</v>
@@ -13251,7 +13381,7 @@
       <c r="H125" s="31"/>
       <c r="I125" s="31"/>
       <c r="J125" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L125" s="31" t="s">
         <v>213</v>
@@ -13292,7 +13422,7 @@
       <c r="H126" s="31"/>
       <c r="I126" s="31"/>
       <c r="J126" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L126" s="31" t="s">
         <v>213</v>
@@ -13333,7 +13463,7 @@
       <c r="H127" s="31"/>
       <c r="I127" s="31"/>
       <c r="J127" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L127" s="31" t="s">
         <v>213</v>
@@ -13374,7 +13504,7 @@
       <c r="H128" s="31"/>
       <c r="I128" s="31"/>
       <c r="J128" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L128" s="31" t="s">
         <v>213</v>
@@ -13415,7 +13545,7 @@
       <c r="H129" s="31"/>
       <c r="I129" s="31"/>
       <c r="J129" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L129" s="31" t="s">
         <v>213</v>
@@ -13456,7 +13586,7 @@
       <c r="H130" s="31"/>
       <c r="I130" s="31"/>
       <c r="J130" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L130" s="31" t="s">
         <v>213</v>
@@ -13497,7 +13627,7 @@
       <c r="H131" s="31"/>
       <c r="I131" s="31"/>
       <c r="J131" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L131" s="31" t="s">
         <v>213</v>
@@ -13538,7 +13668,7 @@
       <c r="H132" s="31"/>
       <c r="I132" s="31"/>
       <c r="J132" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L132" s="31" t="s">
         <v>213</v>
@@ -13579,7 +13709,7 @@
       <c r="H133" s="31"/>
       <c r="I133" s="31"/>
       <c r="J133" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L133" s="31" t="s">
         <v>213</v>
@@ -13620,7 +13750,7 @@
       <c r="H134" s="31"/>
       <c r="I134" s="31"/>
       <c r="J134" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L134" s="31" t="s">
         <v>213</v>
@@ -13661,7 +13791,7 @@
       <c r="H135" s="31"/>
       <c r="I135" s="31"/>
       <c r="J135" s="39" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L135" s="31" t="s">
         <v>213</v>
@@ -13704,7 +13834,7 @@
         <v>183</v>
       </c>
       <c r="J136" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L136" s="31" t="s">
         <v>213</v>
@@ -13745,7 +13875,7 @@
       <c r="H137" s="31"/>
       <c r="I137" s="31"/>
       <c r="J137" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L137" s="31" t="s">
         <v>213</v>
@@ -13786,7 +13916,7 @@
       <c r="H138" s="31"/>
       <c r="I138" s="31"/>
       <c r="J138" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L138" s="31" t="s">
         <v>213</v>
@@ -13827,7 +13957,7 @@
       <c r="H139" s="31"/>
       <c r="I139" s="31"/>
       <c r="J139" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L139" s="31" t="s">
         <v>213</v>
@@ -13868,7 +13998,7 @@
       <c r="H140" s="31"/>
       <c r="I140" s="31"/>
       <c r="J140" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L140" s="31" t="s">
         <v>213</v>
@@ -13909,7 +14039,7 @@
       <c r="H141" s="31"/>
       <c r="I141" s="31"/>
       <c r="J141" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L141" s="31" t="s">
         <v>213</v>
@@ -13950,7 +14080,7 @@
       <c r="H142" s="31"/>
       <c r="I142" s="31"/>
       <c r="J142" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L142" s="31" t="s">
         <v>213</v>
@@ -13991,7 +14121,7 @@
       <c r="H143" s="31"/>
       <c r="I143" s="31"/>
       <c r="J143" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L143" s="31" t="s">
         <v>213</v>
@@ -14032,7 +14162,7 @@
       <c r="H144" s="31"/>
       <c r="I144" s="31"/>
       <c r="J144" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L144" s="31" t="s">
         <v>213</v>
@@ -14073,7 +14203,7 @@
       <c r="H145" s="31"/>
       <c r="I145" s="31"/>
       <c r="J145" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L145" s="31" t="s">
         <v>213</v>
@@ -14114,7 +14244,7 @@
       <c r="H146" s="31"/>
       <c r="I146" s="31"/>
       <c r="J146" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L146" s="31" t="s">
         <v>213</v>
@@ -14155,7 +14285,7 @@
       <c r="H147" s="31"/>
       <c r="I147" s="31"/>
       <c r="J147" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L147" s="31" t="s">
         <v>213</v>
@@ -14196,7 +14326,7 @@
       <c r="H148" s="31"/>
       <c r="I148" s="31"/>
       <c r="J148" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L148" s="31" t="s">
         <v>213</v>
@@ -14237,7 +14367,7 @@
       <c r="H149" s="31"/>
       <c r="I149" s="31"/>
       <c r="J149" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L149" s="31" t="s">
         <v>213</v>
@@ -14278,7 +14408,7 @@
       <c r="H150" s="31"/>
       <c r="I150" s="31"/>
       <c r="J150" s="39" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="L150" s="31" t="s">
         <v>213</v>
@@ -14321,7 +14451,7 @@
         <v>184</v>
       </c>
       <c r="J151" s="39" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L151" s="31" t="s">
         <v>213</v>
@@ -14364,7 +14494,7 @@
         <v>185</v>
       </c>
       <c r="J152" s="39" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L152" s="31" t="s">
         <v>213</v>
@@ -14405,7 +14535,7 @@
       <c r="H153" s="31"/>
       <c r="I153" s="31"/>
       <c r="J153" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L153" s="31" t="s">
         <v>213</v>
@@ -14446,7 +14576,7 @@
       <c r="H154" s="31"/>
       <c r="I154" s="31"/>
       <c r="J154" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L154" s="31" t="s">
         <v>213</v>
@@ -14489,7 +14619,7 @@
         <v>184</v>
       </c>
       <c r="J155" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L155" s="31" t="s">
         <v>213</v>
@@ -14530,7 +14660,7 @@
       <c r="H156" s="31"/>
       <c r="I156" s="31"/>
       <c r="J156" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L156" s="31" t="s">
         <v>213</v>
@@ -14571,7 +14701,7 @@
       <c r="H157" s="31"/>
       <c r="I157" s="31"/>
       <c r="J157" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L157" s="31" t="s">
         <v>213</v>
@@ -14612,7 +14742,7 @@
       <c r="H158" s="31"/>
       <c r="I158" s="31"/>
       <c r="J158" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L158" s="31" t="s">
         <v>213</v>
@@ -14655,7 +14785,7 @@
         <v>17</v>
       </c>
       <c r="J159" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L159" s="31" t="s">
         <v>213</v>
@@ -14696,7 +14826,7 @@
       <c r="H160" s="31"/>
       <c r="I160" s="31"/>
       <c r="J160" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L160" s="31" t="s">
         <v>213</v>
@@ -14737,7 +14867,7 @@
       <c r="H161" s="31"/>
       <c r="I161" s="31"/>
       <c r="J161" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L161" s="31" t="s">
         <v>213</v>
@@ -14778,7 +14908,7 @@
       <c r="H162" s="31"/>
       <c r="I162" s="31"/>
       <c r="J162" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L162" s="31" t="s">
         <v>213</v>
@@ -14819,7 +14949,7 @@
       <c r="H163" s="31"/>
       <c r="I163" s="31"/>
       <c r="J163" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L163" s="31" t="s">
         <v>213</v>
@@ -14862,7 +14992,7 @@
         <v>187</v>
       </c>
       <c r="J164" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L164" s="31" t="s">
         <v>213</v>
@@ -14903,7 +15033,7 @@
       <c r="H165" s="31"/>
       <c r="I165" s="31"/>
       <c r="J165" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L165" s="31" t="s">
         <v>213</v>
@@ -14944,7 +15074,7 @@
       <c r="H166" s="31"/>
       <c r="I166" s="31"/>
       <c r="J166" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L166" s="31" t="s">
         <v>213</v>
@@ -14985,7 +15115,7 @@
       <c r="H167" s="31"/>
       <c r="I167" s="31"/>
       <c r="J167" s="39" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L167" s="31" t="s">
         <v>213</v>
@@ -15026,7 +15156,7 @@
       <c r="H168" s="31"/>
       <c r="I168" s="31"/>
       <c r="J168" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L168" s="31" t="s">
         <v>213</v>
@@ -15069,7 +15199,7 @@
         <v>39</v>
       </c>
       <c r="J169" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L169" s="31" t="s">
         <v>213</v>
@@ -15112,7 +15242,7 @@
         <v>17</v>
       </c>
       <c r="J170" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L170" s="31" t="s">
         <v>213</v>
@@ -15155,7 +15285,7 @@
         <v>188</v>
       </c>
       <c r="J171" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L171" s="31" t="s">
         <v>213</v>
@@ -15196,7 +15326,7 @@
       <c r="H172" s="31"/>
       <c r="I172" s="31"/>
       <c r="J172" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L172" s="31" t="s">
         <v>213</v>
@@ -15239,7 +15369,7 @@
         <v>189</v>
       </c>
       <c r="J173" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L173" s="31" t="s">
         <v>213</v>
@@ -15280,7 +15410,7 @@
       <c r="H174" s="31"/>
       <c r="I174" s="31"/>
       <c r="J174" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L174" s="31" t="s">
         <v>213</v>
@@ -15321,7 +15451,7 @@
       <c r="H175" s="31"/>
       <c r="I175" s="31"/>
       <c r="J175" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L175" s="31" t="s">
         <v>213</v>
@@ -15362,7 +15492,7 @@
       <c r="H176" s="31"/>
       <c r="I176" s="31"/>
       <c r="J176" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L176" s="31" t="s">
         <v>213</v>
@@ -15403,7 +15533,7 @@
       <c r="H177" s="31"/>
       <c r="I177" s="31"/>
       <c r="J177" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L177" s="31" t="s">
         <v>213</v>
@@ -15444,7 +15574,7 @@
       <c r="H178" s="31"/>
       <c r="I178" s="31"/>
       <c r="J178" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L178" s="31" t="s">
         <v>213</v>
@@ -15485,7 +15615,7 @@
       <c r="H179" s="31"/>
       <c r="I179" s="31"/>
       <c r="J179" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L179" s="31" t="s">
         <v>213</v>
@@ -15528,7 +15658,7 @@
         <v>188</v>
       </c>
       <c r="J180" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L180" s="31" t="s">
         <v>213</v>
@@ -15569,7 +15699,7 @@
       <c r="H181" s="31"/>
       <c r="I181" s="31"/>
       <c r="J181" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L181" s="31" t="s">
         <v>213</v>
@@ -15610,7 +15740,7 @@
       <c r="H182" s="31"/>
       <c r="I182" s="31"/>
       <c r="J182" s="39" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L182" s="31" t="s">
         <v>213</v>
@@ -15653,7 +15783,7 @@
         <v>20</v>
       </c>
       <c r="J183" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L183" s="31" t="s">
         <v>213</v>
@@ -15694,7 +15824,7 @@
       <c r="H184" s="31"/>
       <c r="I184" s="31"/>
       <c r="J184" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L184" s="31" t="s">
         <v>213</v>
@@ -15735,7 +15865,7 @@
       <c r="H185" s="31"/>
       <c r="I185" s="31"/>
       <c r="J185" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L185" s="31" t="s">
         <v>213</v>
@@ -15776,7 +15906,7 @@
       <c r="H186" s="31"/>
       <c r="I186" s="31"/>
       <c r="J186" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L186" s="31" t="s">
         <v>213</v>
@@ -15817,7 +15947,7 @@
       <c r="H187" s="31"/>
       <c r="I187" s="31"/>
       <c r="J187" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L187" s="31" t="s">
         <v>213</v>
@@ -15858,7 +15988,7 @@
       <c r="H188" s="31"/>
       <c r="I188" s="31"/>
       <c r="J188" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L188" s="31" t="s">
         <v>213</v>
@@ -15899,7 +16029,7 @@
       <c r="H189" s="31"/>
       <c r="I189" s="31"/>
       <c r="J189" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L189" s="31" t="s">
         <v>213</v>
@@ -15940,7 +16070,7 @@
       <c r="H190" s="31"/>
       <c r="I190" s="31"/>
       <c r="J190" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L190" s="31" t="s">
         <v>213</v>
@@ -15981,7 +16111,7 @@
       <c r="H191" s="31"/>
       <c r="I191" s="31"/>
       <c r="J191" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L191" s="31" t="s">
         <v>213</v>
@@ -16022,7 +16152,7 @@
       <c r="H192" s="31"/>
       <c r="I192" s="31"/>
       <c r="J192" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L192" s="31" t="s">
         <v>213</v>
@@ -16063,7 +16193,7 @@
       <c r="H193" s="31"/>
       <c r="I193" s="31"/>
       <c r="J193" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L193" s="31" t="s">
         <v>213</v>
@@ -16104,7 +16234,7 @@
       <c r="H194" s="31"/>
       <c r="I194" s="31"/>
       <c r="J194" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L194" s="31" t="s">
         <v>213</v>
@@ -16145,7 +16275,7 @@
       <c r="H195" s="31"/>
       <c r="I195" s="31"/>
       <c r="J195" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L195" s="31" t="s">
         <v>213</v>
@@ -16186,7 +16316,7 @@
       <c r="H196" s="31"/>
       <c r="I196" s="31"/>
       <c r="J196" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L196" s="31" t="s">
         <v>213</v>
@@ -16227,7 +16357,7 @@
       <c r="H197" s="31"/>
       <c r="I197" s="31"/>
       <c r="J197" s="39" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L197" s="31" t="s">
         <v>213</v>
@@ -16268,7 +16398,7 @@
       <c r="H198" s="31"/>
       <c r="I198" s="31"/>
       <c r="J198" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L198" s="31" t="s">
         <v>213</v>
@@ -16309,7 +16439,7 @@
       <c r="H199" s="31"/>
       <c r="I199" s="31"/>
       <c r="J199" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L199" s="31" t="s">
         <v>213</v>
@@ -16350,7 +16480,7 @@
       <c r="H200" s="31"/>
       <c r="I200" s="31"/>
       <c r="J200" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L200" s="31" t="s">
         <v>213</v>
@@ -16391,7 +16521,7 @@
       <c r="H201" s="31"/>
       <c r="I201" s="31"/>
       <c r="J201" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L201" s="31" t="s">
         <v>213</v>
@@ -16432,7 +16562,7 @@
       <c r="H202" s="31"/>
       <c r="I202" s="31"/>
       <c r="J202" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L202" s="31" t="s">
         <v>213</v>
@@ -16473,7 +16603,7 @@
       <c r="H203" s="31"/>
       <c r="I203" s="31"/>
       <c r="J203" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L203" s="31" t="s">
         <v>213</v>
@@ -16514,7 +16644,7 @@
       <c r="H204" s="31"/>
       <c r="I204" s="31"/>
       <c r="J204" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L204" s="31" t="s">
         <v>213</v>
@@ -16555,7 +16685,7 @@
       <c r="H205" s="31"/>
       <c r="I205" s="31"/>
       <c r="J205" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L205" s="31" t="s">
         <v>213</v>
@@ -16596,7 +16726,7 @@
       <c r="H206" s="31"/>
       <c r="I206" s="31"/>
       <c r="J206" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L206" s="31" t="s">
         <v>213</v>
@@ -16637,7 +16767,7 @@
       <c r="H207" s="31"/>
       <c r="I207" s="31"/>
       <c r="J207" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L207" s="31" t="s">
         <v>213</v>
@@ -16678,7 +16808,7 @@
       <c r="H208" s="31"/>
       <c r="I208" s="31"/>
       <c r="J208" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L208" s="31" t="s">
         <v>213</v>
@@ -16719,7 +16849,7 @@
       <c r="H209" s="31"/>
       <c r="I209" s="31"/>
       <c r="J209" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L209" s="31" t="s">
         <v>213</v>
@@ -16760,7 +16890,7 @@
       <c r="H210" s="31"/>
       <c r="I210" s="31"/>
       <c r="J210" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L210" s="31" t="s">
         <v>213</v>
@@ -16801,7 +16931,7 @@
       <c r="H211" s="31"/>
       <c r="I211" s="31"/>
       <c r="J211" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L211" s="31" t="s">
         <v>213</v>
@@ -16842,7 +16972,7 @@
       <c r="H212" s="31"/>
       <c r="I212" s="31"/>
       <c r="J212" s="39" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L212" s="31" t="s">
         <v>213</v>
@@ -16883,7 +17013,7 @@
       <c r="H213" s="31"/>
       <c r="I213" s="31"/>
       <c r="J213" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L213" s="31" t="s">
         <v>213</v>
@@ -16924,7 +17054,7 @@
       <c r="H214" s="31"/>
       <c r="I214" s="31"/>
       <c r="J214" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L214" s="31" t="s">
         <v>213</v>
@@ -16965,7 +17095,7 @@
       <c r="H215" s="31"/>
       <c r="I215" s="31"/>
       <c r="J215" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L215" s="31" t="s">
         <v>213</v>
@@ -17006,7 +17136,7 @@
       <c r="H216" s="31"/>
       <c r="I216" s="31"/>
       <c r="J216" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L216" s="31" t="s">
         <v>213</v>
@@ -17047,7 +17177,7 @@
       <c r="H217" s="31"/>
       <c r="I217" s="31"/>
       <c r="J217" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L217" s="31" t="s">
         <v>213</v>
@@ -17088,7 +17218,7 @@
       <c r="H218" s="31"/>
       <c r="I218" s="31"/>
       <c r="J218" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L218" s="31" t="s">
         <v>213</v>
@@ -17129,7 +17259,7 @@
       <c r="H219" s="31"/>
       <c r="I219" s="31"/>
       <c r="J219" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L219" s="31" t="s">
         <v>213</v>
@@ -17170,7 +17300,7 @@
       <c r="H220" s="31"/>
       <c r="I220" s="31"/>
       <c r="J220" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L220" s="31" t="s">
         <v>213</v>
@@ -17210,10 +17340,10 @@
       </c>
       <c r="H221" s="31"/>
       <c r="I221" s="31" t="s">
+        <v>303</v>
+      </c>
+      <c r="J221" s="39" t="s">
         <v>302</v>
-      </c>
-      <c r="J221" s="39" t="s">
-        <v>301</v>
       </c>
       <c r="L221" s="31" t="s">
         <v>213</v>
@@ -17253,10 +17383,10 @@
       </c>
       <c r="H222" s="31"/>
       <c r="I222" s="31" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="J222" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L222" s="31" t="s">
         <v>213</v>
@@ -17299,7 +17429,7 @@
         <v>190</v>
       </c>
       <c r="J223" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L223" s="31" t="s">
         <v>213</v>
@@ -17342,7 +17472,7 @@
         <v>191</v>
       </c>
       <c r="J224" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L224" s="31" t="s">
         <v>213</v>
@@ -17385,7 +17515,7 @@
         <v>192</v>
       </c>
       <c r="J225" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L225" s="31" t="s">
         <v>213</v>
@@ -17428,7 +17558,7 @@
         <v>193</v>
       </c>
       <c r="J226" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L226" s="31" t="s">
         <v>213</v>
@@ -17471,7 +17601,7 @@
         <v>193</v>
       </c>
       <c r="J227" s="39" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L227" s="31" t="s">
         <v>213</v>
@@ -17514,7 +17644,7 @@
         <v>129</v>
       </c>
       <c r="J228" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L228" s="31" t="s">
         <v>213</v>
@@ -17555,7 +17685,7 @@
       <c r="H229" s="31"/>
       <c r="I229" s="31"/>
       <c r="J229" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L229" s="31" t="s">
         <v>213</v>
@@ -17596,7 +17726,7 @@
       <c r="H230" s="31"/>
       <c r="I230" s="31"/>
       <c r="J230" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L230" s="31" t="s">
         <v>213</v>
@@ -17637,7 +17767,7 @@
       <c r="H231" s="31"/>
       <c r="I231" s="31"/>
       <c r="J231" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L231" s="31" t="s">
         <v>213</v>
@@ -17678,7 +17808,7 @@
       <c r="H232" s="31"/>
       <c r="I232" s="31"/>
       <c r="J232" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L232" s="31" t="s">
         <v>213</v>
@@ -17719,7 +17849,7 @@
       <c r="H233" s="31"/>
       <c r="I233" s="31"/>
       <c r="J233" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L233" s="31" t="s">
         <v>213</v>
@@ -17760,7 +17890,7 @@
       <c r="H234" s="31"/>
       <c r="I234" s="31"/>
       <c r="J234" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L234" s="31" t="s">
         <v>213</v>
@@ -17801,7 +17931,7 @@
       <c r="H235" s="31"/>
       <c r="I235" s="31"/>
       <c r="J235" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L235" s="31" t="s">
         <v>213</v>
@@ -17842,7 +17972,7 @@
       <c r="H236" s="31"/>
       <c r="I236" s="31"/>
       <c r="J236" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L236" s="31" t="s">
         <v>213</v>
@@ -17883,7 +18013,7 @@
       <c r="H237" s="31"/>
       <c r="I237" s="31"/>
       <c r="J237" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L237" s="31" t="s">
         <v>213</v>
@@ -17924,7 +18054,7 @@
       <c r="H238" s="31"/>
       <c r="I238" s="31"/>
       <c r="J238" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L238" s="31" t="s">
         <v>213</v>
@@ -17965,7 +18095,7 @@
       <c r="H239" s="31"/>
       <c r="I239" s="31"/>
       <c r="J239" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L239" s="31" t="s">
         <v>213</v>
@@ -18006,7 +18136,7 @@
       <c r="H240" s="31"/>
       <c r="I240" s="31"/>
       <c r="J240" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L240" s="31" t="s">
         <v>213</v>
@@ -18047,7 +18177,7 @@
       <c r="H241" s="31"/>
       <c r="I241" s="31"/>
       <c r="J241" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L241" s="31" t="s">
         <v>213</v>
@@ -18088,7 +18218,7 @@
       <c r="H242" s="31"/>
       <c r="I242" s="31"/>
       <c r="J242" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L242" s="31" t="s">
         <v>213</v>
@@ -18129,7 +18259,7 @@
       <c r="H243" s="31"/>
       <c r="I243" s="31"/>
       <c r="J243" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L243" s="31" t="s">
         <v>213</v>
@@ -18170,7 +18300,7 @@
       <c r="H244" s="31"/>
       <c r="I244" s="31"/>
       <c r="J244" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L244" s="31" t="s">
         <v>213</v>
@@ -18211,7 +18341,7 @@
       <c r="H245" s="31"/>
       <c r="I245" s="31"/>
       <c r="J245" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L245" s="31" t="s">
         <v>213</v>
@@ -18252,7 +18382,7 @@
       <c r="H246" s="31"/>
       <c r="I246" s="31"/>
       <c r="J246" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L246" s="31" t="s">
         <v>213</v>
@@ -18293,7 +18423,7 @@
       <c r="H247" s="31"/>
       <c r="I247" s="31"/>
       <c r="J247" s="39" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L247" s="31" t="s">
         <v>213</v>
@@ -18355,11 +18485,11 @@
       </c>
       <c r="H1" s="31"/>
       <c r="I1" s="31"/>
-      <c r="J1" s="52" t="s">
-        <v>305</v>
-      </c>
-      <c r="K1" s="52" t="s">
-        <v>305</v>
+      <c r="J1" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="K1" s="56" t="s">
+        <v>306</v>
       </c>
       <c r="L1" s="31" t="s">
         <v>213</v>
@@ -18399,11 +18529,11 @@
       </c>
       <c r="H2" s="31"/>
       <c r="I2" s="31"/>
-      <c r="J2" s="52" t="s">
-        <v>305</v>
-      </c>
-      <c r="K2" s="52" t="s">
-        <v>305</v>
+      <c r="J2" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="K2" s="56" t="s">
+        <v>306</v>
       </c>
       <c r="L2" s="31" t="s">
         <v>213</v>

</xml_diff>

<commit_message>
Update notebooks and logfile parsing for April 2025 CB data batch
- Added comprehensive WARP.md project documentation
- Enhanced logfile parsing in src/horse_logic/logfiles.py
- Updated CB notebooks for new data reconciliation and corrections
- Added rbb_28Apr2025 directory with new CB data documentation
- Removed obsolete zip files and duplicate experiment design files
- Updated corrections template workbook

Co-Authored-By: Warp <agent@warp.dev>
</commit_message>
<xml_diff>
--- a/docs/from_CH/Exp1 Errors_Corrections_Template_26Oct2024.xlsx
+++ b/docs/from_CH/Exp1 Errors_Corrections_Template_26Oct2024.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Archived_rows_CSU" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">CBCSU_Times!$A$1:$O$246</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'CSU-RAW'!$A$1:$F$112</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">'CSU-RAW'!$1:$1</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'HD-RAW'!$1:$1</definedName>
@@ -1392,6 +1393,71 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF8E86AE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEEEEEE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF84E291"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF81D41A"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFA6"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1453,6 +1519,10 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1633,7 +1703,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1677,7 +1747,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I133"/>
-  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="10.82"/>
@@ -2725,8 +2795,8 @@
       <c r="G75" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H75" s="0"/>
-      <c r="I75" s="0"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B76" s="2" t="s">
@@ -3204,8 +3274,8 @@
       <c r="G106" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="H106" s="0"/>
-      <c r="I106" s="0"/>
+      <c r="H106" s="11"/>
+      <c r="I106" s="11"/>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B107" s="2" t="s">
@@ -3651,7 +3721,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F112"/>
-  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="2" width="10.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="66.15"/>
@@ -5147,7 +5217,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="12" t="n">
@@ -5345,7 +5415,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P62"/>
-  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="23" width="14.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="23" width="11.6"/>
@@ -8041,11 +8111,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+  <sheetPr filterMode="true">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O1048576"/>
-  <sheetFormatPr defaultColWidth="10.515625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.515625" defaultRowHeight="12.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="23" width="14.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="23" width="11.6"/>
@@ -8062,7 +8132,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="23" width="10.51"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
         <v>198</v>
       </c>
@@ -8109,7 +8179,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8152,7 +8222,7 @@
         <v>GO, 10.93</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8195,7 +8265,7 @@
         <v>GO, 11.81</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8238,7 +8308,7 @@
         <v>GO, 6.24</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8281,7 +8351,7 @@
         <v>GO, 18.08</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8324,7 +8394,7 @@
         <v>GO, 9.29</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8367,7 +8437,7 @@
         <v>GO, 12.82</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8408,7 +8478,7 @@
         <v>GO, 12.45</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8449,7 +8519,7 @@
         <v>GO, 11.97</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8490,7 +8560,7 @@
         <v>GO, 26.66</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8531,7 +8601,7 @@
         <v>GO, 12.27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8572,7 +8642,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8613,7 +8683,7 @@
         <v>GO, 11.52</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8654,7 +8724,7 @@
         <v>GO, 12.93</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8695,7 +8765,7 @@
         <v>GO, 11.6</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8736,7 +8806,7 @@
         <v>GO, 13.14</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8777,7 +8847,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8818,7 +8888,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8859,7 +8929,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8900,7 +8970,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8941,7 +9011,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="n">
         <v>45246</v>
       </c>
@@ -8982,7 +9052,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="30" t="n">
         <v>45246</v>
       </c>
@@ -9023,7 +9093,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="30" t="n">
         <v>45246</v>
       </c>
@@ -9064,7 +9134,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="30" t="n">
         <v>45246</v>
       </c>
@@ -9105,7 +9175,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="30" t="n">
         <v>45246</v>
       </c>
@@ -9189,7 +9259,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9232,7 +9302,7 @@
         <v>GO, 28.2</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9273,7 +9343,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9314,7 +9384,7 @@
         <v>GO, 10.07</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9355,7 +9425,7 @@
         <v>GO, 13.74</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9396,7 +9466,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9437,7 +9507,7 @@
         <v>GO, 10.08</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9478,7 +9548,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9519,7 +9589,7 @@
         <v>GO, 10.46</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9560,7 +9630,7 @@
         <v>GO, 11.93</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9601,7 +9671,7 @@
         <v>GO, 11.33</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9642,7 +9712,7 @@
         <v>GO, 10.93</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9683,7 +9753,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="30" t="n">
         <v>45247</v>
       </c>
@@ -9726,7 +9796,7 @@
         <v>GO, 11.6</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="30" t="n">
         <v>45248</v>
       </c>
@@ -9772,7 +9842,7 @@
         <v>GO, 27.2</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="30" t="n">
         <v>45248</v>
       </c>
@@ -9816,7 +9886,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="30" t="n">
         <v>45248</v>
       </c>
@@ -9862,7 +9932,7 @@
         <v>GO, 11.66</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="30" t="n">
         <v>45248</v>
       </c>
@@ -9908,7 +9978,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="43" t="n">
         <v>45248</v>
       </c>
@@ -9952,7 +10022,7 @@
         <v>GO, 9.35</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="30" t="n">
         <v>45248</v>
       </c>
@@ -9993,7 +10063,7 @@
         <v>GO, 9.15</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10034,7 +10104,7 @@
         <v>GO, 9.01</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10075,7 +10145,7 @@
         <v>GO, 8.95</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10116,7 +10186,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10157,7 +10227,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10198,7 +10268,7 @@
         <v>GO, 8.69</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10239,7 +10309,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10280,7 +10350,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10321,7 +10391,7 @@
         <v>GO, 9.09</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10362,7 +10432,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10403,7 +10473,7 @@
         <v>GO, 9.13</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="30" t="n">
         <v>45249</v>
       </c>
@@ -10446,7 +10516,7 @@
         <v>GO, 10.68</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10492,7 +10562,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="30" t="n">
         <v>45248</v>
       </c>
@@ -10535,7 +10605,7 @@
         <v>GO, 12.4</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="30" t="n">
         <v>45249</v>
       </c>
@@ -10578,7 +10648,7 @@
         <v>GO, 10.52</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="30" t="n">
         <v>45249</v>
       </c>
@@ -10621,7 +10691,7 @@
         <v>GO, 10.22</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="30" t="n">
         <v>45249</v>
       </c>
@@ -10664,7 +10734,7 @@
         <v>GO, 7.83</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="30" t="n">
         <v>45249</v>
       </c>
@@ -10707,7 +10777,7 @@
         <v>GO, 12.04</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="30" t="n">
         <v>45250</v>
       </c>
@@ -10748,7 +10818,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="30" t="n">
         <v>45250</v>
       </c>
@@ -10791,7 +10861,7 @@
         <v>GO, 12.6</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="30" t="n">
         <v>45250</v>
       </c>
@@ -10835,7 +10905,7 @@
         <v>GO, 9.68</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="30" t="n">
         <v>45250</v>
       </c>
@@ -10879,7 +10949,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="30" t="n">
         <v>45250</v>
       </c>
@@ -10923,7 +10993,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="30" t="n">
         <v>45250</v>
       </c>
@@ -10966,7 +11036,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11640,7 +11710,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="86" s="53" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="86" s="53" customFormat="true" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11684,7 +11754,7 @@
         <v>GO, 10.12</v>
       </c>
     </row>
-    <row r="87" s="53" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="87" s="53" customFormat="true" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="30" t="n">
         <v>45251</v>
       </c>
@@ -11728,7 +11798,7 @@
         <v>GO, 9.49</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="30" t="n">
         <v>45252</v>
       </c>
@@ -11771,7 +11841,7 @@
         <v>GO, 29.46</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="30" t="n">
         <v>45253</v>
       </c>
@@ -11814,7 +11884,7 @@
         <v>GO, 10.93</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="30" t="n">
         <v>45253</v>
       </c>
@@ -11857,7 +11927,7 @@
         <v>GO, 11.85</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="30" t="n">
         <v>45253</v>
       </c>
@@ -11898,7 +11968,7 @@
         <v>GO, 18.88</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="30" t="n">
         <v>45253</v>
       </c>
@@ -11939,7 +12009,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="30" t="n">
         <v>45253</v>
       </c>
@@ -11980,7 +12050,7 @@
         <v>GO, 10.94</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12021,7 +12091,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12062,7 +12132,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12103,7 +12173,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12144,7 +12214,7 @@
         <v>GO, 11.93</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12185,7 +12255,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12226,7 +12296,7 @@
         <v>GO, 10.48</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12269,7 +12339,7 @@
         <v>GO, 12.67</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12310,7 +12380,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12351,7 +12421,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="30" t="n">
         <v>45253</v>
       </c>
@@ -12392,7 +12462,7 @@
         <v>GO, 12.8</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="30" t="n">
         <v>45253</v>
       </c>
@@ -13677,7 +13747,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13720,7 +13790,7 @@
         <v>GO, 9.29</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13761,7 +13831,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13802,7 +13872,7 @@
         <v>GO, 10.36</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13843,7 +13913,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13884,7 +13954,7 @@
         <v>GO, 9.87</v>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13925,7 +13995,7 @@
         <v>GO, 9.33</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="30" t="n">
         <v>45256</v>
       </c>
@@ -13966,7 +14036,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14007,7 +14077,7 @@
         <v>GO, 8.76</v>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14048,7 +14118,7 @@
         <v>GO, 9.22</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14089,7 +14159,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14130,7 +14200,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14171,7 +14241,7 @@
         <v>GO, 9.43</v>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14212,7 +14282,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14253,7 +14323,7 @@
         <v>GO, 9.66</v>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="30" t="n">
         <v>45256</v>
       </c>
@@ -14294,7 +14364,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14337,7 +14407,7 @@
         <v>GO, 27.17</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14380,7 +14450,7 @@
         <v>GO, 11.2</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14421,7 +14491,7 @@
         <v>GO, 10.14</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14462,7 +14532,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14505,7 +14575,7 @@
         <v>GO, 10.79</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14546,7 +14616,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14587,7 +14657,7 @@
         <v>GO, 9.87</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14628,7 +14698,7 @@
         <v>GO, 10.87</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14671,7 +14741,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14712,7 +14782,7 @@
         <v>GO, 10.13</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14753,7 +14823,7 @@
         <v>GO, 10.22</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14794,7 +14864,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14835,7 +14905,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14878,7 +14948,7 @@
         <v>GO, 10.87</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14919,7 +14989,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="30" t="n">
         <v>45257</v>
       </c>
@@ -14960,7 +15030,7 @@
         <v>GO, 10.87</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15001,7 +15071,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15042,7 +15112,7 @@
         <v>GO, 7.99</v>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15085,7 +15155,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15128,7 +15198,7 @@
         <v>GO, 9.14</v>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15171,7 +15241,7 @@
         <v>GO, 18.01</v>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15212,7 +15282,7 @@
         <v>GO, 10.56</v>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15255,7 +15325,7 @@
         <v>GO, 9.22</v>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15296,7 +15366,7 @@
         <v>GO, 9.55</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15337,7 +15407,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15378,7 +15448,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15419,7 +15489,7 @@
         <v>GO, 10.13</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15460,7 +15530,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15501,7 +15571,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15544,7 +15614,7 @@
         <v>GO, 9.63</v>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15585,7 +15655,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15626,7 +15696,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15669,7 +15739,7 @@
         <v>GO, 8.23</v>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15710,7 +15780,7 @@
         <v>GO, 25.39</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15751,7 +15821,7 @@
         <v>GO, 8.16</v>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15792,7 +15862,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15833,7 +15903,7 @@
         <v>GO, 9.48</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15874,7 +15944,7 @@
         <v>GO, 8.82</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15915,7 +15985,7 @@
         <v>GO, 9.14</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15956,7 +16026,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="30" t="n">
         <v>45257</v>
       </c>
@@ -15997,7 +16067,7 @@
         <v>GO, 8.6</v>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16038,7 +16108,7 @@
         <v>GO, 8.95</v>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16079,7 +16149,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16120,7 +16190,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16161,7 +16231,7 @@
         <v>GO, 9.08</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16202,7 +16272,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16243,7 +16313,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16284,7 +16354,7 @@
         <v>GO, 7.62</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16325,7 +16395,7 @@
         <v>GO, 15.96</v>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16366,7 +16436,7 @@
         <v>GO, 8.56</v>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16407,7 +16477,7 @@
         <v>GO, 11.54</v>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16448,7 +16518,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16489,7 +16559,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16530,7 +16600,7 @@
         <v>GO, 8.61</v>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16571,7 +16641,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16612,7 +16682,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16653,7 +16723,7 @@
         <v>GO, 9.6</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16694,7 +16764,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16735,7 +16805,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16776,7 +16846,7 @@
         <v>GO, 8.46</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16817,7 +16887,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="30" t="n">
         <v>45257</v>
       </c>
@@ -16858,7 +16928,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="30" t="n">
         <v>45258</v>
       </c>
@@ -16899,7 +16969,7 @@
         <v>GO, 10.12</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="30" t="n">
         <v>45258</v>
       </c>
@@ -16940,7 +17010,7 @@
         <v>GO, 19.18</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="30" t="n">
         <v>45258</v>
       </c>
@@ -16981,7 +17051,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17022,7 +17092,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17063,7 +17133,7 @@
         <v>GO, 9.92</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17104,7 +17174,7 @@
         <v>GO, 9.49</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17145,7 +17215,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17186,7 +17256,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17229,7 +17299,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17272,7 +17342,7 @@
         <v>GO, 19.61</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17315,7 +17385,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17358,7 +17428,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17401,7 +17471,7 @@
         <v>GO, 8.87</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17444,7 +17514,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="30" t="n">
         <v>45258</v>
       </c>
@@ -17487,7 +17557,7 @@
         <v>GO, 8.09</v>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17530,7 +17600,7 @@
         <v>GO, 11.13</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17571,7 +17641,7 @@
         <v>GO, 12.67</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17612,7 +17682,7 @@
         <v>GO, 11.73</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17653,7 +17723,7 @@
         <v>GO, 14</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17694,7 +17764,7 @@
         <v>GO, 12.4</v>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17735,7 +17805,7 @@
         <v>GO, 12.94</v>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17776,7 +17846,7 @@
         <v>GO, 12.37</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17817,7 +17887,7 @@
         <v>GO, 26.7</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17858,7 +17928,7 @@
         <v>GO, 16.89</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17899,7 +17969,7 @@
         <v>GO, 11.99</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17940,7 +18010,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="238" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="30" t="n">
         <v>45247</v>
       </c>
@@ -17981,7 +18051,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18022,7 +18092,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18063,7 +18133,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A241" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18104,7 +18174,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A242" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18145,7 +18215,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A243" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18186,7 +18256,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A244" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18227,7 +18297,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A245" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18268,7 +18338,7 @@
         <v>NOGO, 30</v>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="15.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A246" s="30" t="n">
         <v>45247</v>
       </c>
@@ -18314,6 +18384,13 @@
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <autoFilter ref="A1:O246">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Nix"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -18321,6 +18398,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -18330,7 +18408,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="30" t="n">

</xml_diff>